<commit_message>
trend screener update 2026-09-28 23:59 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -3163,12 +3163,12 @@
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>0921.HK</t>
+          <t>1913.HK</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>海信家电</t>
+          <t>普拉达</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
@@ -3183,21 +3183,21 @@
       </c>
       <c r="E44" s="8" t="inlineStr"/>
       <c r="F44" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>21.2</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>1913.HK</t>
+          <t>0921.HK</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>普拉达</t>
+          <t>海信家电</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
@@ -3212,10 +3212,10 @@
       </c>
       <c r="E45" s="8" t="inlineStr"/>
       <c r="F45" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>38.9</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="46">
@@ -3395,12 +3395,12 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>1579.HK</t>
+          <t>2648.HK</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>颐海国际</t>
+          <t>安井食品</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3415,21 +3415,21 @@
       </c>
       <c r="E52" s="4" t="inlineStr"/>
       <c r="F52" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>13.76</v>
+        <v>63.55</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>2648.HK</t>
+          <t>1579.HK</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>安井食品</t>
+          <t>颐海国际</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -3444,10 +3444,10 @@
       </c>
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>63.55</v>
+        <v>13.76</v>
       </c>
     </row>
     <row r="54">
@@ -4004,12 +4004,12 @@
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>0116.HK</t>
+          <t>1836.HK</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>周生生</t>
+          <t>九兴控股</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -4024,21 +4024,21 @@
       </c>
       <c r="E73" s="8" t="inlineStr"/>
       <c r="F73" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G73" s="8" t="n">
-        <v>12.72</v>
+        <v>12.03</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>1836.HK</t>
+          <t>0116.HK</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>九兴控股</t>
+          <t>周生生</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
@@ -4053,10 +4053,10 @@
       </c>
       <c r="E74" s="8" t="inlineStr"/>
       <c r="F74" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G74" s="8" t="n">
-        <v>12.03</v>
+        <v>12.72</v>
       </c>
     </row>
     <row r="75">
@@ -4120,12 +4120,12 @@
     <row r="77">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>2607.HK</t>
+          <t>2273.HK</t>
         </is>
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>上海医药</t>
+          <t>固生堂</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
@@ -4140,21 +4140,21 @@
       </c>
       <c r="E77" s="9" t="inlineStr"/>
       <c r="F77" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G77" s="9" t="n">
-        <v>10.82</v>
+        <v>27.46</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>2273.HK</t>
+          <t>2607.HK</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>固生堂</t>
+          <t>上海医药</t>
         </is>
       </c>
       <c r="C78" s="9" t="inlineStr">
@@ -4169,68 +4169,68 @@
       </c>
       <c r="E78" s="9" t="inlineStr"/>
       <c r="F78" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G78" s="9" t="n">
-        <v>27.46</v>
+        <v>10.82</v>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="A79" s="10" t="inlineStr">
+        <is>
+          <t>2378.HK</t>
+        </is>
+      </c>
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>保诚</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E79" s="10" t="inlineStr"/>
+      <c r="F79" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G79" s="10" t="n">
+        <v>98.40000000000001</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>6067.HK</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>星源材质</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr"/>
-      <c r="F79" s="2" t="n">
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G79" s="2" t="n">
+      <c r="G80" s="2" t="n">
         <v>6.97</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="10" t="inlineStr">
-        <is>
-          <t>2378.HK</t>
-        </is>
-      </c>
-      <c r="B80" s="10" t="inlineStr">
-        <is>
-          <t>保诚</t>
-        </is>
-      </c>
-      <c r="C80" s="10" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D80" s="10" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E80" s="10" t="inlineStr"/>
-      <c r="F80" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="G80" s="10" t="n">
-        <v>98.40000000000001</v>
       </c>
     </row>
     <row r="81">

</xml_diff>

<commit_message>
trend screener update 2026-10-13 00:42 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -520,7 +520,7 @@
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>食品饮料调味品/酒</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>食物饮品</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>食品饮料调味品/酒</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>原材料</t>
+          <t>化工</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>食物饮品</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>食物饮品</t>
+          <t>食品饮料</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>黄金及贵金属</t>
+          <t>贵金属</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -2601,12 +2601,12 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>6030.HK</t>
+          <t>0388.HK</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>中信证券</t>
+          <t>香港交易所</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2621,21 +2621,21 @@
       </c>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>23.8</v>
+        <v>375.4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>0388.HK</t>
+          <t>6030.HK</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>香港交易所</t>
+          <t>中信证券</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2650,10 +2650,10 @@
       </c>
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>375.4</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="37">
@@ -2918,61 +2918,61 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>3690.HK</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>美团-W</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>1024.HK</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>快手-W</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr"/>
-      <c r="F46" s="6" t="n">
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G46" s="6" t="n">
+      <c r="G47" s="6" t="n">
         <v>29.26</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>3690.HK</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>美团-W</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G47" s="2" t="n">
-        <v>71.8</v>
       </c>
     </row>
     <row r="48">
@@ -4840,7 +4840,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>扫描日期：2026-10-12</t>
+          <t>扫描日期：2026-10-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
trend screener update 2026-10-13 08:52 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -49,12 +49,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0F2F1"/>
-        <bgColor rgb="00E0F2F1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE4EC"/>
         <bgColor rgb="00FCE4EC"/>
       </patternFill>
@@ -79,6 +73,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00ECEFF1"/>
+        <bgColor rgb="00ECEFF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F3E5F5"/>
         <bgColor rgb="00F3E5F5"/>
       </patternFill>
@@ -97,8 +97,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ECEFF1"/>
-        <bgColor rgb="00ECEFF1"/>
+        <fgColor rgb="00E0F2F1"/>
+        <bgColor rgb="00E0F2F1"/>
       </patternFill>
     </fill>
     <fill>
@@ -514,13 +514,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
@@ -584,22 +584,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>1313.HK</t>
+          <t>1364.HK</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>华润建材科技</t>
+          <t>古茗</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>建筑</t>
+          <t>消费服务</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -613,541 +613,629 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.97</v>
+        <v>23.16</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.925</v>
+        <v>22.776</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>-1.02</v>
+        <v>4.28</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-4.55</v>
+        <v>-0.52</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>1364.HK</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>古茗</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>0116.HK</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>周生生</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>专业零售</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>13.27</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>13.097</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>1.49</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>0921.HK</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>海信家电</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>耐用品</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>22.22</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>21.448</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>-1.01</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>0027.HK</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>银河娱乐</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>消费服务</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>23.02</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>22.762</v>
-      </c>
-      <c r="I3" s="3" t="n">
-        <v>4.21</v>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>-0.52</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>0116.HK</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>周生生</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="G5" s="2" t="n">
+        <v>32.74</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>31.238</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>-3.15</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>-1.67</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>0175.HK</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>吉利汽车</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>专业零售</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>汽车</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>13.097</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>1.49</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>0027.HK</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>银河娱乐</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>消费服务</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="G6" s="2" t="n">
+        <v>15.56</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>14.95</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>-6.05</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>-0.68</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>0268.HK</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>金蝶国际</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>软件服务</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
-        <v>32.68</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>31.232</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>-3.17</v>
-      </c>
-      <c r="J5" s="3" t="n">
-        <v>-1.67</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>0268.HK</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>金蝶国际</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="G7" s="3" t="n">
+        <v>8.525</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>7.579</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>-6.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>7687.HK</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>易控智驾</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>软件服务</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G6" s="4" t="n">
-        <v>8.555</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>7.583</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>-6.4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>7687.HK</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>易控智驾</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>软件服务</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="G8" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>66.315</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>-6.21</v>
+      </c>
+      <c r="J8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>3618.HK</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>重庆农村商业银行</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>中国银行</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G7" s="4" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>66.205</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>-6.36</v>
-      </c>
-      <c r="J7" s="4" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>3618.HK</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>重庆农村商业银行</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>中国银行</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="G9" s="4" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>6.321</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>1579.HK</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>颐海国际</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>食品饮料</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n">
-        <v>6.605</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>6.324</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>1579.HK</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>颐海国际</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="G10" s="5" t="n">
+        <v>14.81</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>14.202</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>0220.HK</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>统一企业中国</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>食品饮料</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>14.87</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>14.208</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>1.75</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>0220.HK</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>统一企业中国</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="G11" s="5" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>7.227</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>-0.78</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>3319.HK</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>雅生活服务</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>中国地产&amp;物管</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>1.945</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>-3.02</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>2768.HK</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>国恩科技</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>化工</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>37.52</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>40.028</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>14.84</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>0772.HK</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>阅文集团</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>互联网</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>20.311</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>-5.68</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>6979.HK</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>珍酒李渡</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>食品饮料</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>7.54</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>7.221</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>3.48</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>-0.78</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>2768.HK</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>国恩科技</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>化工</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>SOS-C</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>8.029</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>0345.HK</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>维他奶国际</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>食品饮料</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>37.42</v>
-      </c>
-      <c r="H11" s="7" t="n">
-        <v>40.018</v>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>-4.62</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>14.84</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>0772.HK</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>阅文集团</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>互联网</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>21.66</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>20.307</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>4.45</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>-5.68</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>6979.HK</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>珍酒李渡</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>食品饮料</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>SOS-C</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
-        <v>8.414999999999999</v>
-      </c>
-      <c r="H13" s="6" t="n">
-        <v>8.029999999999999</v>
-      </c>
-      <c r="I13" s="6" t="n">
-        <v>4.01</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>-0.23</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>0345.HK</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>维他奶国际</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>食品饮料</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>SOS-C</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="n">
+      <c r="G16" s="5" t="n">
         <v>6.825</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H16" s="5" t="n">
         <v>6.755</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I16" s="5" t="n">
         <v>2.89</v>
       </c>
-      <c r="J14" s="6" t="n">
+      <c r="J16" s="5" t="n">
         <v>0.28</v>
       </c>
     </row>
@@ -1273,16 +1361,16 @@
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>59.95</v>
+        <v>60</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>58.565</v>
+        <v>58.57</v>
       </c>
       <c r="I2" s="9" t="n">
-        <v>13.42</v>
+        <v>13.43</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>52.328</v>
+        <v>52.329</v>
       </c>
       <c r="K2" s="9" t="n"/>
       <c r="L2" s="9" t="n">
@@ -1321,16 +1409,16 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>34.78</v>
+        <v>36.8</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>34.338</v>
+        <v>34.54</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1.45</v>
+        <v>2.04</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>34.1</v>
+        <v>34.133</v>
       </c>
       <c r="K3" s="7" t="n"/>
       <c r="L3" s="7" t="n">
@@ -1369,19 +1457,19 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>145.7</v>
+        <v>146.3</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>141.56</v>
+        <v>141.62</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>-5.85</v>
+        <v>-5.81</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>141.457</v>
+        <v>141.467</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="L4" s="7" t="n">
         <v>3</v>
@@ -1448,34 +1536,34 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>1333.HK</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>博雷顿</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>-36.4</v>
-      </c>
-      <c r="F2" s="2" t="n">
+      <c r="E2" s="10" t="n">
+        <v>-35.5</v>
+      </c>
+      <c r="F2" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>12.72</v>
+      <c r="G2" s="10" t="n">
+        <v>12.9</v>
       </c>
     </row>
     <row r="3">
@@ -1500,13 +1588,13 @@
         </is>
       </c>
       <c r="E3" s="9" t="n">
-        <v>-31.5</v>
+        <v>-31.68</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>43.74</v>
+        <v>43.62</v>
       </c>
     </row>
     <row r="4">
@@ -1531,44 +1619,44 @@
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-29.8</v>
+        <v>-29.92</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>55.95</v>
+        <v>55.85</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>2556.HK</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>迈富时</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>-29.62</v>
-      </c>
-      <c r="F5" s="4" t="n">
+      <c r="E5" s="3" t="n">
+        <v>-29.59</v>
+      </c>
+      <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="4" t="n">
-        <v>47.58</v>
+      <c r="G5" s="3" t="n">
+        <v>47.6</v>
       </c>
     </row>
     <row r="6">
@@ -1593,261 +1681,261 @@
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>-28.12</v>
+        <v>-27.64</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>35.32</v>
+        <v>35.56</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>6951.HK</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>三环集团</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
-        <v>-26.01</v>
-      </c>
-      <c r="F7" s="2" t="n">
+      <c r="E7" s="10" t="n">
+        <v>-25.72</v>
+      </c>
+      <c r="F7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>103</v>
+      <c r="G7" s="10" t="n">
+        <v>103.4</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>6166.HK</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>剑桥科技</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>-24.54</v>
-      </c>
-      <c r="F8" s="4" t="n">
+      <c r="E8" s="3" t="n">
+        <v>-24.78</v>
+      </c>
+      <c r="F8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="4" t="n">
-        <v>95.3</v>
+      <c r="G8" s="3" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>0668.HK</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>安克创新</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n">
-        <v>-21.43</v>
-      </c>
-      <c r="F9" s="3" t="n">
+      <c r="E9" s="2" t="n">
+        <v>-22.88</v>
+      </c>
+      <c r="F9" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="3" t="n">
-        <v>108.2</v>
+      <c r="G9" s="2" t="n">
+        <v>106.2</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>0631.HK</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>三一国际</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n">
-        <v>-21.32</v>
-      </c>
-      <c r="F10" s="2" t="n">
+      <c r="E10" s="10" t="n">
+        <v>-21.61</v>
+      </c>
+      <c r="F10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>8.01</v>
+      <c r="G10" s="10" t="n">
+        <v>7.98</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>2382.HK</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>舜宇光学科技</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="3" t="n">
         <v>-18.15</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="3" t="n">
         <v>58.85</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>1316.HK</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>耐世特</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n">
-        <v>-17.99</v>
-      </c>
-      <c r="F12" s="3" t="n">
+      <c r="E12" s="2" t="n">
+        <v>-17.33</v>
+      </c>
+      <c r="F12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="3" t="n">
-        <v>4.4</v>
+      <c r="G12" s="2" t="n">
+        <v>4.435</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>0992.HK</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>联想集团</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
-        <v>-17.62</v>
-      </c>
-      <c r="F13" s="4" t="n">
+      <c r="E13" s="3" t="n">
+        <v>-17.24</v>
+      </c>
+      <c r="F13" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="4" t="n">
-        <v>30.96</v>
+      <c r="G13" s="3" t="n">
+        <v>31.1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>0038.HK</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>第一拖拉机股份</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n">
-        <v>-17.19</v>
-      </c>
-      <c r="F14" s="2" t="n">
+      <c r="E14" s="10" t="n">
+        <v>-16.62</v>
+      </c>
+      <c r="F14" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>8.115</v>
+      <c r="G14" s="10" t="n">
+        <v>8.17</v>
       </c>
     </row>
     <row r="15">
@@ -1872,105 +1960,105 @@
         </is>
       </c>
       <c r="E15" s="9" t="n">
-        <v>-16.35</v>
+        <v>-16.26</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>91.84999999999999</v>
+        <v>91.95</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>2676.HK</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>纳芯微</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="3" t="n">
         <v>-15.89</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F16" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="G16" s="3" t="n">
         <v>153.5</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>2419.HK</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>德康农牧</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n">
-        <v>-14.76</v>
-      </c>
-      <c r="F17" s="6" t="n">
+      <c r="E17" s="5" t="n">
+        <v>-15.16</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="6" t="n">
-        <v>52.85</v>
+      <c r="G17" s="5" t="n">
+        <v>52.6</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>0669.HK</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>创科实业</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="10" t="n">
         <v>-14.26</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F18" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G18" s="10" t="n">
         <v>125.4</v>
       </c>
     </row>
@@ -1996,44 +2084,44 @@
         </is>
       </c>
       <c r="E19" s="8" t="n">
-        <v>-13.77</v>
+        <v>-12.95</v>
       </c>
       <c r="F19" s="8" t="n">
         <v>2</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>11.65</v>
+        <v>11.76</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>2202.HK</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>万科企业</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E20" s="10" t="n">
-        <v>-11.74</v>
-      </c>
-      <c r="F20" s="10" t="n">
+      <c r="E20" s="6" t="n">
+        <v>-11.57</v>
+      </c>
+      <c r="F20" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="10" t="n">
-        <v>2.48</v>
+      <c r="G20" s="6" t="n">
+        <v>2.485</v>
       </c>
     </row>
     <row r="21">
@@ -2058,86 +2146,86 @@
         </is>
       </c>
       <c r="E21" s="9" t="n">
-        <v>-11.66</v>
+        <v>-11.49</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>51.15</v>
+        <v>51.25</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>2714.HK</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>牧原股份</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n">
-        <v>-10.83</v>
-      </c>
-      <c r="F22" s="6" t="n">
+      <c r="E22" s="5" t="n">
+        <v>-11.13</v>
+      </c>
+      <c r="F22" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="G22" s="6" t="n">
-        <v>35.56</v>
+      <c r="G22" s="5" t="n">
+        <v>35.44</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>3347.HK</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>泰格医药</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>3800.HK</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>协鑫科技</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E23" s="9" t="n">
-        <v>-10.47</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <v>42.22</v>
+      <c r="E23" s="3" t="n">
+        <v>-10.76</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>0.705</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>9688.HK</t>
+          <t>3347.HK</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>再鼎医药</t>
+          <t>泰格医药</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -2151,44 +2239,44 @@
         </is>
       </c>
       <c r="E24" s="9" t="n">
-        <v>-10.4</v>
+        <v>-10.31</v>
       </c>
       <c r="F24" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>18.96</v>
+        <v>42.3</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>3800.HK</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>协鑫科技</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>9688.HK</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>再鼎医药</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n">
-        <v>-10.13</v>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>0.71</v>
+      <c r="E25" s="9" t="n">
+        <v>-10.26</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>18.99</v>
       </c>
     </row>
     <row r="26">
@@ -2244,168 +2332,168 @@
         </is>
       </c>
       <c r="E27" s="9" t="n">
-        <v>-9.970000000000001</v>
+        <v>-9.630000000000001</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>5.33</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>0013.HK</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>和黄医药</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>21.16</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>0839.HK</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>中教控股</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="n">
+        <v>-7.21</v>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>1.93</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>2888.HK</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>渣打集团</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>-6.81</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>229.8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>2390.HK</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>知乎-W</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E28" s="8" t="n">
-        <v>-8.859999999999999</v>
-      </c>
-      <c r="F28" s="8" t="n">
+      <c r="E31" s="8" t="n">
+        <v>-6.74</v>
+      </c>
+      <c r="F31" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G28" s="8" t="n">
-        <v>8.795</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>0013.HK</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>和黄医药</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="G31" s="8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>0293.HK</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>国泰航空</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E29" s="9" t="n">
-        <v>-7.57</v>
-      </c>
-      <c r="F29" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="9" t="n">
-        <v>21.26</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>0839.HK</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>中教控股</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>-7.21</v>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>1.93</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>2888.HK</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>渣打集团</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="n">
-        <v>-6.89</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G31" s="5" t="n">
-        <v>229.6</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>0293.HK</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>国泰航空</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>-6.36</v>
-      </c>
-      <c r="F32" s="2" t="n">
+      <c r="E32" s="10" t="n">
+        <v>-6.15</v>
+      </c>
+      <c r="F32" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="G32" s="2" t="n">
-        <v>13.92</v>
+      <c r="G32" s="10" t="n">
+        <v>13.95</v>
       </c>
     </row>
     <row r="33">
@@ -2430,13 +2518,13 @@
         </is>
       </c>
       <c r="E33" s="9" t="n">
-        <v>-5.87</v>
+        <v>-6.05</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>1</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>214.8</v>
+        <v>214.4</v>
       </c>
     </row>
     <row r="34">
@@ -2461,421 +2549,421 @@
         </is>
       </c>
       <c r="E34" s="9" t="n">
-        <v>-4.85</v>
+        <v>-5.12</v>
       </c>
       <c r="F34" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="9" t="n">
-        <v>208</v>
+        <v>207.4</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>1788.HK</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>国泰君安国际</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="E35" s="4" t="n">
         <v>-1.2</v>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="4" t="n">
         <v>2.875</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>1299.HK</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>友邦保险</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr"/>
-      <c r="F36" s="5" t="n">
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G36" s="5" t="n">
-        <v>72.95</v>
+      <c r="G36" s="4" t="n">
+        <v>73.05</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>2628.HK</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>中国人寿</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr"/>
-      <c r="F37" s="5" t="n">
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G37" s="5" t="n">
-        <v>25.56</v>
+      <c r="G37" s="4" t="n">
+        <v>25.62</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>1336.HK</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>新华保险</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr"/>
-      <c r="F38" s="5" t="n">
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G38" s="5" t="n">
-        <v>43.82</v>
+      <c r="G38" s="4" t="n">
+        <v>43.9</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>1339.HK</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>中国人民保险集团</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr"/>
-      <c r="F39" s="5" t="n">
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G39" s="5" t="n">
-        <v>5.18</v>
+      <c r="G39" s="4" t="n">
+        <v>5.21</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>0966.HK</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>中国太平</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr"/>
-      <c r="F40" s="5" t="n">
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G40" s="5" t="n">
-        <v>17.98</v>
+      <c r="G40" s="4" t="n">
+        <v>18.01</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>0388.HK</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>香港交易所</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr"/>
-      <c r="F41" s="5" t="n">
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G41" s="5" t="n">
-        <v>379.2</v>
+      <c r="G41" s="4" t="n">
+        <v>379.6</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>6030.HK</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>中信证券</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr"/>
-      <c r="F42" s="5" t="n">
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G42" s="5" t="n">
+      <c r="G42" s="4" t="n">
         <v>23.74</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>6886.HK</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>华泰证券</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr"/>
-      <c r="F43" s="5" t="n">
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G43" s="5" t="n">
-        <v>16.27</v>
+      <c r="G43" s="4" t="n">
+        <v>16.28</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>6099.HK</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>招商证券</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr"/>
-      <c r="F44" s="5" t="n">
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G44" s="5" t="n">
-        <v>13.9</v>
+      <c r="G44" s="4" t="n">
+        <v>13.89</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>6066.HK</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>中信建投证券</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="5" t="n">
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G45" s="5" t="n">
-        <v>11.14</v>
+      <c r="G45" s="4" t="n">
+        <v>11.19</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="10" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>1109.HK</t>
         </is>
       </c>
-      <c r="B46" s="10" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>华润置地</t>
         </is>
       </c>
-      <c r="C46" s="10" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="D46" s="10" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E46" s="10" t="inlineStr"/>
-      <c r="F46" s="10" t="n">
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr"/>
+      <c r="F46" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G46" s="10" t="n">
+      <c r="G46" s="6" t="n">
         <v>30.54</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="10" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>0817.HK</t>
         </is>
       </c>
-      <c r="B47" s="10" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>中国金茂</t>
         </is>
       </c>
-      <c r="C47" s="10" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E47" s="10" t="inlineStr"/>
-      <c r="F47" s="10" t="n">
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G47" s="10" t="n">
+      <c r="G47" s="6" t="n">
         <v>1.28</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="10" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>1113.HK</t>
         </is>
       </c>
-      <c r="B48" s="10" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>长实集团</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="D48" s="10" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E48" s="10" t="inlineStr"/>
-      <c r="F48" s="10" t="n">
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr"/>
+      <c r="F48" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G48" s="10" t="n">
-        <v>45.06</v>
+      <c r="G48" s="6" t="n">
+        <v>45.2</v>
       </c>
     </row>
     <row r="49">
@@ -2904,35 +2992,35 @@
         <v>2</v>
       </c>
       <c r="G49" s="11" t="n">
-        <v>29.84</v>
+        <v>29.94</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>0257.HK</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>光大环境</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="n">
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="inlineStr"/>
+      <c r="F50" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="G50" s="2" t="n">
+      <c r="G50" s="10" t="n">
         <v>4.635</v>
       </c>
     </row>
@@ -2962,7 +3050,7 @@
         <v>4</v>
       </c>
       <c r="G51" s="11" t="n">
-        <v>77.65000000000001</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52">
@@ -2991,297 +3079,297 @@
         <v>2</v>
       </c>
       <c r="G52" s="8" t="n">
-        <v>29.1</v>
+        <v>29.16</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>9618.HK</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>京东集团-SW</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr"/>
-      <c r="F53" s="3" t="n">
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G53" s="3" t="n">
-        <v>105.2</v>
+      <c r="G53" s="2" t="n">
+        <v>104.9</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>9927.HK</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>赛力斯</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr"/>
-      <c r="F54" s="3" t="n">
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G54" s="3" t="n">
-        <v>38.28</v>
+      <c r="G54" s="2" t="n">
+        <v>37.76</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>3808.HK</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>中国重汽</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr"/>
-      <c r="F55" s="2" t="n">
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr"/>
+      <c r="F55" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="G55" s="2" t="n">
-        <v>34.7</v>
+      <c r="G55" s="10" t="n">
+        <v>35.04</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>2020.HK</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>安踏体育</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr"/>
-      <c r="F56" s="3" t="n">
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G56" s="3" t="n">
-        <v>72.05</v>
+      <c r="G56" s="2" t="n">
+        <v>72.45</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>3998.HK</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>波司登</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr"/>
-      <c r="F57" s="3" t="n">
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G57" s="3" t="n">
-        <v>4.285</v>
+      <c r="G57" s="2" t="n">
+        <v>4.295</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>1913.HK</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>普拉达</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr"/>
-      <c r="F58" s="3" t="n">
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G58" s="3" t="n">
-        <v>37.4</v>
+      <c r="G58" s="2" t="n">
+        <v>37.78</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>1929.HK</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>周大福</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr"/>
-      <c r="F59" s="3" t="n">
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G59" s="3" t="n">
-        <v>10.71</v>
+      <c r="G59" s="2" t="n">
+        <v>10.74</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>6181.HK</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>老铺黄金</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="inlineStr"/>
-      <c r="F60" s="3" t="n">
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G60" s="3" t="n">
-        <v>312.6</v>
+      <c r="G60" s="2" t="n">
+        <v>314.8</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>1928.HK</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>金沙中国有限公司</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr"/>
-      <c r="F61" s="3" t="n">
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G61" s="3" t="n">
-        <v>11.37</v>
+      <c r="G61" s="2" t="n">
+        <v>11.42</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>1128.HK</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>永利澳门</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr"/>
-      <c r="F62" s="3" t="n">
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G62" s="3" t="n">
-        <v>5.01</v>
+      <c r="G62" s="2" t="n">
+        <v>5.025</v>
       </c>
     </row>
     <row r="63">
@@ -3310,123 +3398,123 @@
         <v>4</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>5.195</v>
+        <v>5.215</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="inlineStr">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>9980.HK</t>
         </is>
       </c>
-      <c r="B64" s="6" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>东鹏饮料</t>
         </is>
       </c>
-      <c r="C64" s="6" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="inlineStr"/>
-      <c r="F64" s="6" t="n">
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr"/>
+      <c r="F64" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G64" s="6" t="n">
-        <v>98.8</v>
+      <c r="G64" s="5" t="n">
+        <v>98.55</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="inlineStr">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>9858.HK</t>
         </is>
       </c>
-      <c r="B65" s="6" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>优然牧业</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr"/>
-      <c r="F65" s="6" t="n">
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr"/>
+      <c r="F65" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G65" s="6" t="n">
+      <c r="G65" s="5" t="n">
         <v>3.46</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>2367.HK</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B66" s="5" t="inlineStr">
         <is>
           <t>巨子生物</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr"/>
-      <c r="F66" s="6" t="n">
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr"/>
+      <c r="F66" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G66" s="6" t="n">
-        <v>23.18</v>
+      <c r="G66" s="5" t="n">
+        <v>23.14</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="inlineStr">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>2698.HK</t>
         </is>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>乐舒适</t>
         </is>
       </c>
-      <c r="C67" s="6" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="inlineStr"/>
-      <c r="F67" s="6" t="n">
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr"/>
+      <c r="F67" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G67" s="6" t="n">
-        <v>25.88</v>
+      <c r="G67" s="5" t="n">
+        <v>25.78</v>
       </c>
     </row>
     <row r="68">
@@ -3459,90 +3547,90 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="A69" s="10" t="inlineStr">
         <is>
           <t>2057.HK</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B69" s="10" t="inlineStr">
         <is>
           <t>中通快递-W</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C69" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr"/>
-      <c r="F69" s="2" t="n">
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E69" s="10" t="inlineStr"/>
+      <c r="F69" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="G69" s="2" t="n">
-        <v>161.7</v>
+      <c r="G69" s="10" t="n">
+        <v>162.1</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" s="10" t="inlineStr">
         <is>
           <t>6936.HK</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B70" s="10" t="inlineStr">
         <is>
           <t>顺丰控股</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C70" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr"/>
-      <c r="F70" s="2" t="n">
+      <c r="D70" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E70" s="10" t="inlineStr"/>
+      <c r="F70" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="G70" s="2" t="n">
-        <v>29.24</v>
+      <c r="G70" s="10" t="n">
+        <v>29.42</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" s="10" t="inlineStr">
         <is>
           <t>0001.HK</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B71" s="10" t="inlineStr">
         <is>
           <t>长和</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C71" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr"/>
-      <c r="F71" s="2" t="n">
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E71" s="10" t="inlineStr"/>
+      <c r="F71" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="G71" s="2" t="n">
-        <v>66.95</v>
+      <c r="G71" s="10" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="72">
@@ -3571,152 +3659,152 @@
         <v>2</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>18.4</v>
+        <v>18.47</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="inlineStr">
+      <c r="A73" s="3" t="inlineStr">
         <is>
           <t>6809.HK</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>澜起科技</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C73" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr"/>
-      <c r="F73" s="4" t="n">
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr"/>
+      <c r="F73" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G73" s="4" t="n">
-        <v>242</v>
+      <c r="G73" s="3" t="n">
+        <v>241.8</v>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="4" t="inlineStr">
+      <c r="A74" s="3" t="inlineStr">
         <is>
           <t>0981.HK</t>
         </is>
       </c>
-      <c r="B74" s="4" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>中芯国际</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
+      <c r="C74" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr"/>
-      <c r="F74" s="4" t="n">
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr"/>
+      <c r="F74" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G74" s="4" t="n">
+      <c r="G74" s="3" t="n">
         <v>55.55</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="4" t="inlineStr">
+      <c r="A75" s="3" t="inlineStr">
         <is>
           <t>2018.HK</t>
         </is>
       </c>
-      <c r="B75" s="4" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>瑞声科技</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr"/>
-      <c r="F75" s="4" t="n">
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr"/>
+      <c r="F75" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G75" s="4" t="n">
+      <c r="G75" s="3" t="n">
         <v>36.56</v>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="4" t="inlineStr">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>1810.HK</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>小米集团-W</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr"/>
+      <c r="F76" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G76" s="3" t="n">
+        <v>25.04</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>0501.HK</t>
         </is>
       </c>
-      <c r="B76" s="4" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>豪威集团</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr"/>
-      <c r="F76" s="4" t="n">
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr"/>
+      <c r="F77" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G76" s="4" t="n">
+      <c r="G77" s="3" t="n">
         <v>65.8</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>1810.HK</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>小米集团-W</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr"/>
-      <c r="F77" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G77" s="4" t="n">
-        <v>25</v>
       </c>
     </row>
     <row r="78">
@@ -3745,7 +3833,7 @@
         <v>3</v>
       </c>
       <c r="G78" s="9" t="n">
-        <v>53</v>
+        <v>53.4</v>
       </c>
     </row>
     <row r="79">
@@ -3774,210 +3862,210 @@
         <v>1</v>
       </c>
       <c r="G79" s="9" t="n">
-        <v>31.6</v>
+        <v>31.54</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="4" t="inlineStr">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>1304.HK</t>
         </is>
       </c>
-      <c r="B80" s="4" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>峰岹科技</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
+      <c r="C80" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E80" s="4" t="inlineStr"/>
-      <c r="F80" s="4" t="n">
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr"/>
+      <c r="F80" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G80" s="4" t="n">
-        <v>108.8</v>
+      <c r="G80" s="3" t="n">
+        <v>108.7</v>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="inlineStr">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <t>6818.HK</t>
         </is>
       </c>
-      <c r="B81" s="5" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
         <is>
           <t>中国光大银行</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="C81" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr"/>
-      <c r="F81" s="5" t="n">
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G81" s="5" t="n">
-        <v>2.825</v>
+      <c r="G81" s="4" t="n">
+        <v>2.83</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="A82" s="10" t="inlineStr">
         <is>
           <t>0868.HK</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B82" s="10" t="inlineStr">
         <is>
           <t>信义玻璃</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C82" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr"/>
-      <c r="F82" s="2" t="n">
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E82" s="10" t="inlineStr"/>
+      <c r="F82" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="G82" s="2" t="n">
-        <v>8.074999999999999</v>
+      <c r="G82" s="10" t="n">
+        <v>8.07</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="inlineStr">
+      <c r="A83" s="3" t="inlineStr">
         <is>
           <t>1729.HK</t>
         </is>
       </c>
-      <c r="B83" s="4" t="inlineStr">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>汇聚科技</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
+      <c r="C83" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr"/>
-      <c r="F83" s="4" t="n">
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr"/>
+      <c r="F83" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G83" s="4" t="n">
-        <v>13.88</v>
+      <c r="G83" s="3" t="n">
+        <v>13.96</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>1836.HK</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>九兴控股</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E84" s="3" t="inlineStr"/>
-      <c r="F84" s="3" t="n">
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G84" s="3" t="n">
-        <v>12.45</v>
+      <c r="G84" s="2" t="n">
+        <v>12.49</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="10" t="inlineStr">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>0823.HK</t>
         </is>
       </c>
-      <c r="B85" s="10" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>领展房产基金</t>
         </is>
       </c>
-      <c r="C85" s="10" t="inlineStr">
+      <c r="C85" s="6" t="inlineStr">
         <is>
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="D85" s="10" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E85" s="10" t="inlineStr"/>
-      <c r="F85" s="10" t="n">
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr"/>
+      <c r="F85" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="G85" s="10" t="n">
-        <v>37.72</v>
+      <c r="G85" s="6" t="n">
+        <v>37.76</v>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="6" t="inlineStr">
+      <c r="A86" s="5" t="inlineStr">
         <is>
           <t>1610.HK</t>
         </is>
       </c>
-      <c r="B86" s="6" t="inlineStr">
+      <c r="B86" s="5" t="inlineStr">
         <is>
           <t>中粮家佳康</t>
         </is>
       </c>
-      <c r="C86" s="6" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E86" s="6" t="inlineStr"/>
-      <c r="F86" s="6" t="n">
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr"/>
+      <c r="F86" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G86" s="6" t="n">
-        <v>1.08</v>
+      <c r="G86" s="5" t="n">
+        <v>1.07</v>
       </c>
     </row>
     <row r="87">
@@ -4006,36 +4094,36 @@
         <v>2</v>
       </c>
       <c r="G87" s="9" t="n">
-        <v>11.09</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="inlineStr">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>2378.HK</t>
         </is>
       </c>
-      <c r="B88" s="5" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>保诚</t>
         </is>
       </c>
-      <c r="C88" s="5" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr"/>
-      <c r="F88" s="5" t="n">
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr"/>
+      <c r="F88" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G88" s="5" t="n">
-        <v>94.05</v>
+      <c r="G88" s="4" t="n">
+        <v>93.84999999999999</v>
       </c>
     </row>
     <row r="89">
@@ -4068,32 +4156,32 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="inlineStr">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>2518.HK</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>汽车之家-S</t>
         </is>
       </c>
-      <c r="C90" s="3" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D90" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E90" s="3" t="inlineStr"/>
-      <c r="F90" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G90" s="3" t="n">
-        <v>40</v>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>39.02</v>
       </c>
     </row>
     <row r="91">
@@ -4122,7 +4210,7 @@
         <v>3</v>
       </c>
       <c r="G91" s="8" t="n">
-        <v>0.058</v>
+        <v>0.059</v>
       </c>
     </row>
     <row r="92">
@@ -4151,7 +4239,7 @@
         <v>4</v>
       </c>
       <c r="G92" s="9" t="n">
-        <v>4.48</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="93">
@@ -4180,7 +4268,7 @@
         <v>4</v>
       </c>
       <c r="G93" s="9" t="n">
-        <v>10.8</v>
+        <v>10.72</v>
       </c>
     </row>
     <row r="94">
@@ -4209,7 +4297,7 @@
         <v>1</v>
       </c>
       <c r="G94" s="9" t="n">
-        <v>10.35</v>
+        <v>10.39</v>
       </c>
     </row>
     <row r="95">
@@ -4238,94 +4326,94 @@
         <v>1</v>
       </c>
       <c r="G95" s="9" t="n">
-        <v>7.02</v>
+        <v>7.045</v>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="10" t="inlineStr">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>6049.HK</t>
         </is>
       </c>
-      <c r="B96" s="10" t="inlineStr">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>保利物业</t>
         </is>
       </c>
-      <c r="C96" s="10" t="inlineStr">
+      <c r="C96" s="6" t="inlineStr">
         <is>
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="D96" s="10" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E96" s="10" t="inlineStr"/>
-      <c r="F96" s="10" t="n">
+      <c r="D96" s="6" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="inlineStr"/>
+      <c r="F96" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G96" s="10" t="n">
-        <v>27.6</v>
+      <c r="G96" s="6" t="n">
+        <v>27.62</v>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="inlineStr">
+      <c r="A97" s="10" t="inlineStr">
         <is>
           <t>1191.HK</t>
         </is>
       </c>
-      <c r="B97" s="2" t="inlineStr">
+      <c r="B97" s="10" t="inlineStr">
         <is>
           <t>海光芯正</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr">
+      <c r="C97" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr"/>
-      <c r="F97" s="2" t="n">
+      <c r="D97" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E97" s="10" t="inlineStr"/>
+      <c r="F97" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="G97" s="2" t="n">
-        <v>106.5</v>
+      <c r="G97" s="10" t="n">
+        <v>107.1</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="4" t="inlineStr">
+      <c r="A98" s="3" t="inlineStr">
         <is>
           <t>3268.HK</t>
         </is>
       </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B98" s="3" t="inlineStr">
         <is>
           <t>美格智能</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C98" s="3" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D98" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E98" s="4" t="inlineStr"/>
-      <c r="F98" s="4" t="n">
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr"/>
+      <c r="F98" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G98" s="4" t="n">
-        <v>15.18</v>
+      <c r="G98" s="3" t="n">
+        <v>15.17</v>
       </c>
     </row>
     <row r="99">
@@ -4354,35 +4442,35 @@
         <v>4</v>
       </c>
       <c r="G99" s="8" t="n">
-        <v>5.145</v>
+        <v>5.155</v>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr">
+      <c r="A100" s="10" t="inlineStr">
         <is>
           <t>0548.HK</t>
         </is>
       </c>
-      <c r="B100" s="2" t="inlineStr">
+      <c r="B100" s="10" t="inlineStr">
         <is>
           <t>深圳高速公路股份</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
+      <c r="C100" s="10" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr"/>
-      <c r="F100" s="2" t="n">
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="inlineStr"/>
+      <c r="F100" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="G100" s="2" t="n">
+      <c r="G100" s="10" t="n">
         <v>6.66</v>
       </c>
     </row>
@@ -4412,7 +4500,7 @@
         <v>3</v>
       </c>
       <c r="G101" s="11" t="n">
-        <v>2.095</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="102">
@@ -4441,7 +4529,7 @@
         <v>1</v>
       </c>
       <c r="G102" s="11" t="n">
-        <v>1.62</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="103">
@@ -4466,13 +4554,13 @@
         </is>
       </c>
       <c r="E103" s="7" t="n">
-        <v>-29.6</v>
+        <v>-29.09</v>
       </c>
       <c r="F103" s="7" t="n">
         <v>12</v>
       </c>
       <c r="G103" s="7" t="n">
-        <v>17.74</v>
+        <v>17.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
trend screener update 2026-10-13 10:06 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -2708,12 +2708,12 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>0966.HK</t>
+          <t>0388.HK</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>中国太平</t>
+          <t>香港交易所</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2728,21 +2728,21 @@
       </c>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>18.01</v>
+        <v>379.6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>0388.HK</t>
+          <t>0966.HK</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>香港交易所</t>
+          <t>中国太平</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2757,10 +2757,10 @@
       </c>
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>379.6</v>
+        <v>18.01</v>
       </c>
     </row>
     <row r="42">
@@ -3752,12 +3752,12 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>1810.HK</t>
+          <t>0501.HK</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>小米集团-W</t>
+          <t>豪威集团</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3775,18 +3775,18 @@
         <v>2</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>25.04</v>
+        <v>65.8</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>0501.HK</t>
+          <t>1810.HK</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>豪威集团</t>
+          <t>小米集团-W</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -3804,7 +3804,7 @@
         <v>2</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>65.8</v>
+        <v>25.04</v>
       </c>
     </row>
     <row r="78">

</xml_diff>

<commit_message>
trend screener update 2026-10-13 13:27 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -836,7 +836,7 @@
         <v>8.525</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>7.579</v>
+        <v>7.58</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>0.96</v>
@@ -1230,7 +1230,7 @@
         <v>6.825</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>6.755</v>
+        <v>6.756</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>2.89</v>
@@ -2708,12 +2708,12 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>0388.HK</t>
+          <t>0966.HK</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>香港交易所</t>
+          <t>中国太平</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2728,21 +2728,21 @@
       </c>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>379.6</v>
+        <v>18.01</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>0966.HK</t>
+          <t>6030.HK</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>中国太平</t>
+          <t>中信证券</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2757,21 +2757,21 @@
       </c>
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>18.01</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>6030.HK</t>
+          <t>0388.HK</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>中信证券</t>
+          <t>香港交易所</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2786,10 +2786,10 @@
       </c>
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>23.74</v>
+        <v>379.6</v>
       </c>
     </row>
     <row r="43">
@@ -3373,61 +3373,61 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>9980.HK</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>东鹏饮料</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr"/>
+      <c r="F63" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="5" t="n">
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
         <is>
           <t>2689.HK</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>玖龙纸业</t>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr"/>
-      <c r="F63" s="7" t="n">
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr"/>
+      <c r="F64" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G63" s="7" t="n">
+      <c r="G64" s="7" t="n">
         <v>5.215</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>9980.HK</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>东鹏饮料</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr"/>
-      <c r="F64" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G64" s="5" t="n">
-        <v>98.55</v>
       </c>
     </row>
     <row r="65">
@@ -3723,12 +3723,12 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>2018.HK</t>
+          <t>1810.HK</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>瑞声科技</t>
+          <t>小米集团-W</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -3743,21 +3743,21 @@
       </c>
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>36.56</v>
+        <v>25.04</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>0501.HK</t>
+          <t>2018.HK</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>豪威集团</t>
+          <t>瑞声科技</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3772,21 +3772,21 @@
       </c>
       <c r="E76" s="3" t="inlineStr"/>
       <c r="F76" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>65.8</v>
+        <v>36.56</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>1810.HK</t>
+          <t>0501.HK</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>小米集团-W</t>
+          <t>豪威集团</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -3804,7 +3804,7 @@
         <v>2</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>25.04</v>
+        <v>65.8</v>
       </c>
     </row>
     <row r="78">

</xml_diff>

<commit_message>
trend screener update 2026-10-13 13:55 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -2621,12 +2621,12 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>2628.HK</t>
+          <t>1336.HK</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>中国人寿</t>
+          <t>新华保险</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -2644,18 +2644,18 @@
         <v>4</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>25.62</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>1336.HK</t>
+          <t>2628.HK</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>新华保险</t>
+          <t>中国人寿</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -2673,7 +2673,7 @@
         <v>4</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>43.9</v>
+        <v>25.62</v>
       </c>
     </row>
     <row r="39">
@@ -2708,12 +2708,12 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>0966.HK</t>
+          <t>0388.HK</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>中国太平</t>
+          <t>香港交易所</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2728,21 +2728,21 @@
       </c>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>18.01</v>
+        <v>379.6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>6030.HK</t>
+          <t>0966.HK</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>中信证券</t>
+          <t>中国太平</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2757,21 +2757,21 @@
       </c>
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>23.74</v>
+        <v>18.01</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>0388.HK</t>
+          <t>6030.HK</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>香港交易所</t>
+          <t>中信证券</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2786,10 +2786,10 @@
       </c>
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>379.6</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="43">
@@ -3373,61 +3373,61 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>2689.HK</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>玖龙纸业</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr"/>
+      <c r="F63" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>5.215</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>9980.HK</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>东鹏饮料</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr"/>
-      <c r="F63" s="5" t="n">
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr"/>
+      <c r="F64" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G63" s="5" t="n">
+      <c r="G64" s="5" t="n">
         <v>98.55</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>2689.HK</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>玖龙纸业</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D64" s="7" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr"/>
-      <c r="F64" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="G64" s="7" t="n">
-        <v>5.215</v>
       </c>
     </row>
     <row r="65">
@@ -3723,12 +3723,12 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>1810.HK</t>
+          <t>2018.HK</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>小米集团-W</t>
+          <t>瑞声科技</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -3743,21 +3743,21 @@
       </c>
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>25.04</v>
+        <v>36.56</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>2018.HK</t>
+          <t>1810.HK</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>瑞声科技</t>
+          <t>小米集团-W</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3772,10 +3772,10 @@
       </c>
       <c r="E76" s="3" t="inlineStr"/>
       <c r="F76" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>36.56</v>
+        <v>25.04</v>
       </c>
     </row>
     <row r="77">

</xml_diff>

<commit_message>
trend screener update 2026-10-13 14:14 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -2621,12 +2621,12 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>1336.HK</t>
+          <t>2628.HK</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>新华保险</t>
+          <t>中国人寿</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -2644,18 +2644,18 @@
         <v>4</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>43.9</v>
+        <v>25.62</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2628.HK</t>
+          <t>1336.HK</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>中国人寿</t>
+          <t>新华保险</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -2673,7 +2673,7 @@
         <v>4</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>25.62</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="39">
@@ -2708,12 +2708,12 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>0388.HK</t>
+          <t>0966.HK</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>香港交易所</t>
+          <t>中国太平</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2728,21 +2728,21 @@
       </c>
       <c r="E40" s="4" t="inlineStr"/>
       <c r="F40" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>379.6</v>
+        <v>18.01</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>0966.HK</t>
+          <t>0388.HK</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>中国太平</t>
+          <t>香港交易所</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2757,10 +2757,10 @@
       </c>
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>18.01</v>
+        <v>379.6</v>
       </c>
     </row>
     <row r="42">
@@ -3433,12 +3433,12 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>9858.HK</t>
+          <t>2367.HK</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>优然牧业</t>
+          <t>巨子生物</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -3453,21 +3453,21 @@
       </c>
       <c r="E65" s="5" t="inlineStr"/>
       <c r="F65" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>3.46</v>
+        <v>23.14</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>2367.HK</t>
+          <t>9858.HK</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>巨子生物</t>
+          <t>优然牧业</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -3482,10 +3482,10 @@
       </c>
       <c r="E66" s="5" t="inlineStr"/>
       <c r="F66" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>23.14</v>
+        <v>3.46</v>
       </c>
     </row>
     <row r="67">
@@ -3752,12 +3752,12 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>1810.HK</t>
+          <t>0501.HK</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>小米集团-W</t>
+          <t>豪威集团</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3775,18 +3775,18 @@
         <v>2</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>25.04</v>
+        <v>65.8</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>0501.HK</t>
+          <t>1810.HK</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>豪威集团</t>
+          <t>小米集团-W</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -3804,7 +3804,7 @@
         <v>2</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>65.8</v>
+        <v>25.04</v>
       </c>
     </row>
     <row r="78">

</xml_diff>

<commit_message>
trend screener update 2026-10-13 19:31 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -2737,12 +2737,12 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>0388.HK</t>
+          <t>6030.HK</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>香港交易所</t>
+          <t>中信证券</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2757,21 +2757,21 @@
       </c>
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>379.6</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>6030.HK</t>
+          <t>0388.HK</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>中信证券</t>
+          <t>香港交易所</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2786,10 +2786,10 @@
       </c>
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>23.74</v>
+        <v>379.6</v>
       </c>
     </row>
     <row r="43">
@@ -3433,12 +3433,12 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>2367.HK</t>
+          <t>9858.HK</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>巨子生物</t>
+          <t>优然牧业</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -3453,21 +3453,21 @@
       </c>
       <c r="E65" s="5" t="inlineStr"/>
       <c r="F65" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>23.14</v>
+        <v>3.46</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>9858.HK</t>
+          <t>2367.HK</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>优然牧业</t>
+          <t>巨子生物</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -3482,10 +3482,10 @@
       </c>
       <c r="E66" s="5" t="inlineStr"/>
       <c r="F66" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>3.46</v>
+        <v>23.14</v>
       </c>
     </row>
     <row r="67">
@@ -3752,12 +3752,12 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>0501.HK</t>
+          <t>1810.HK</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>豪威集团</t>
+          <t>小米集团-W</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3775,18 +3775,18 @@
         <v>2</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>65.8</v>
+        <v>25.04</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>1810.HK</t>
+          <t>0501.HK</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>小米集团-W</t>
+          <t>豪威集团</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -3804,7 +3804,7 @@
         <v>2</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>25.04</v>
+        <v>65.8</v>
       </c>
     </row>
     <row r="78">

</xml_diff>

<commit_message>
trend screener update 2026-10-15 11:39 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -34,7 +34,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +107,12 @@
         <bgColor rgb="00FBE9E7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+        <bgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -134,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -149,6 +155,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -514,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -613,16 +620,16 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1.02</v>
+        <v>1.025</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0.9419999999999999</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.24</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-4.47</v>
+        <v>-4.46</v>
       </c>
     </row>
     <row r="3">
@@ -657,544 +664,806 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>39.08</v>
+        <v>38.78</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>41.186</v>
+        <v>41.156</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-3.34</v>
+        <v>-3.41</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>-1.87</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>0116.HK</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>周生生</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>专业零售</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1377.HK</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>鼎泰高科</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>工业工程</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>13.12</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>13.183</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>1.52</v>
-      </c>
+      <c r="G4" s="2" t="n">
+        <v>199.3</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>235.85</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>-14.45</v>
+      </c>
+      <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>9896.HK</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>名创优品</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>零售</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>20.56</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>18.508</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>-6.49</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>0116.HK</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>周生生</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>专业零售</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>13.07</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>13.178</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>1.51</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
           <t>0027.HK</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>银河娱乐</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>消费服务</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
-        <v>32.88</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>31.524</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>-1.73</v>
-      </c>
-      <c r="J5" s="3" t="n">
+      <c r="G7" s="3" t="n">
+        <v>33.28</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>31.564</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="J7" s="3" t="n">
         <v>-1.63</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>0268.HK</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>金蝶国际</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>软件服务</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G6" s="4" t="n">
-        <v>8.175000000000001</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>7.745</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="J6" s="4" t="n">
+      <c r="G8" s="4" t="n">
+        <v>8.185</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>7.746</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>-6.33</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>3320.HK</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>华润医药</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Health Care</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>药品及生物科技</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n">
-        <v>4.62</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>4.404</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>-0.16</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="G9" s="5" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>4.414</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>3618.HK</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>重庆农村商业银行</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>中国银行</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n">
-        <v>6.505</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>6.383</v>
-      </c>
-      <c r="I8" s="6" t="n">
-        <v>1.69</v>
-      </c>
-      <c r="J8" s="6" t="n">
+      <c r="G10" s="6" t="n">
+        <v>6.545</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>6.386</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J10" s="6" t="n">
         <v>0.7</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>0220.HK</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>统一企业中国</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>食品饮料</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G9" s="7" t="n">
-        <v>7.66</v>
-      </c>
-      <c r="H9" s="7" t="n">
-        <v>7.367</v>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J9" s="7" t="n">
+      <c r="G11" s="7" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>7.371</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="J11" s="7" t="n">
         <v>-0.68</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>1579.HK</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>颐海国际</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>食品饮料</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G12" s="7" t="n">
         <v>14.87</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H12" s="7" t="n">
         <v>14.391</v>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="I12" s="7" t="n">
         <v>5.31</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="J12" s="7" t="n">
         <v>1.81</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>3319.HK</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>雅生活服务</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>中国地产&amp;物管</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>9985.HK</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>卫龙美味</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>食品饮料</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>SOS-B</t>
         </is>
       </c>
-      <c r="G11" s="8" t="n">
-        <v>2.015</v>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>1.786</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>9.91</v>
-      </c>
-      <c r="J11" s="8" t="n">
-        <v>-2.77</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>2768.HK</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>国恩科技</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>化工</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>30.34</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>37.996</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>-9.74</v>
-      </c>
-      <c r="J12" s="9" t="n">
-        <v>14.3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>0772.HK</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>阅文集团</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>互联网</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>SETUP_OK</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>SOS-B</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="n">
-        <v>22.54</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>20.763</v>
-      </c>
-      <c r="I13" s="10" t="n">
-        <v>5.34</v>
-      </c>
-      <c r="J13" s="10" t="n">
-        <v>-5.5</v>
+      <c r="G13" s="7" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>6.559</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>-4.04</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
+          <t>0241.HK</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>阿里健康</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>互联网药店</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>2.848</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>-5.26</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>3319.HK</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>雅生活服务</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>中国地产&amp;物管</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>2.015</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>1.786</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>-2.77</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>2768.HK</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>国恩科技</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>化工</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>29.48</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>37.91</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>-9.949999999999999</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>14.28</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>0772.HK</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>阅文集团</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>互联网</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>22.18</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>20.727</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>-5.51</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>1310.HK</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>香港宽频</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>电讯</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>6.015</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>5.741</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>-0.97</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>9899.HK</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>网易云音乐</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>媒体及娱乐</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>SETUP_OK</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>SOS-B</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>84.75</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>83.605</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>-7.84</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
           <t>6979.HK</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>珍酒李渡</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>食品饮料</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>SOS-C</t>
         </is>
       </c>
-      <c r="G14" s="7" t="n">
-        <v>8.515000000000001</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>8.154</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>4.68</v>
-      </c>
-      <c r="J14" s="7" t="n">
+      <c r="G20" s="7" t="n">
+        <v>8.535</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>8.156000000000001</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="J20" s="7" t="n">
         <v>-0.03</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>0956.HK</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>新天绿色能源</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>Utilities</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>公用事业</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>SETUP_OK</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>SOS-C</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>3.335</v>
-      </c>
-      <c r="H15" s="11" t="n">
-        <v>3.335</v>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="J15" s="11" t="n">
-        <v>-1.8</v>
+      <c r="G21" s="11" t="n">
+        <v>3.315</v>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>3.333</v>
+      </c>
+      <c r="I21" s="11" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J21" s="11" t="n">
+        <v>-1.81</v>
       </c>
     </row>
   </sheetData>
@@ -1319,16 +1588,16 @@
         </is>
       </c>
       <c r="G2" s="5" t="n">
-        <v>54.75</v>
+        <v>53.6</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>58.335</v>
+        <v>58.22</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>9.449999999999999</v>
+        <v>9.23</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>52.446</v>
+        <v>52.427</v>
       </c>
       <c r="K2" s="5" t="n"/>
       <c r="L2" s="5" t="n">
@@ -1367,16 +1636,16 @@
         </is>
       </c>
       <c r="G3" s="9" t="n">
-        <v>33.5</v>
+        <v>34</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>34.666</v>
+        <v>34.716</v>
       </c>
       <c r="I3" s="9" t="n">
-        <v>2.25</v>
+        <v>2.39</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>34.434</v>
+        <v>34.442</v>
       </c>
       <c r="K3" s="9" t="n"/>
       <c r="L3" s="9" t="n">
@@ -1415,19 +1684,19 @@
         </is>
       </c>
       <c r="G4" s="9" t="n">
-        <v>142.2</v>
+        <v>143.5</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>142.44</v>
+        <v>142.57</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>-2.9</v>
+        <v>-2.81</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>142.546</v>
+        <v>142.568</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="L4" s="9" t="n">
         <v>5</v>
@@ -1494,65 +1763,65 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>6166.HK</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>剑桥科技</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>2315.HK</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>百奥赛图-B</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>-36.51</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>50.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2556.HK</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>迈富时</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>-37.73</v>
-      </c>
-      <c r="F2" s="4" t="n">
+      <c r="E3" s="4" t="n">
+        <v>-35.74</v>
+      </c>
+      <c r="F3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G2" s="4" t="n">
-        <v>78.65000000000001</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>2315.HK</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>百奥赛图-B</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>-37.08</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>50.15</v>
+      <c r="G3" s="4" t="n">
+        <v>43.44</v>
       </c>
     </row>
     <row r="4">
@@ -1577,24 +1846,24 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-35.33</v>
+        <v>-35.69</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>3</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>31.78</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2556.HK</t>
+          <t>6166.HK</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>迈富时</t>
+          <t>剑桥科技</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1608,13 +1877,13 @@
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-34.76</v>
+        <v>-35.39</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>44.1</v>
+        <v>81.59999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -1639,75 +1908,75 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-33.51</v>
+        <v>-32.72</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>92.55</v>
+        <v>93.65000000000001</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>0992.HK</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>联想集团</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>-30.87</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>25.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>1333.HK</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>博雷顿</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
-        <v>-33.4</v>
-      </c>
-      <c r="F7" s="2" t="n">
+      <c r="E8" s="2" t="n">
+        <v>-29.65</v>
+      </c>
+      <c r="F8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>13.32</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>0992.HK</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>联想集团</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>-31.4</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>25.78</v>
+      <c r="G8" s="2" t="n">
+        <v>14.07</v>
       </c>
     </row>
     <row r="9">
@@ -1732,13 +2001,13 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-27.01</v>
+        <v>-26.67</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>7.43</v>
+        <v>7.465</v>
       </c>
     </row>
     <row r="10">
@@ -1763,199 +2032,199 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-26.16</v>
+        <v>-26.55</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>29.98</v>
+        <v>29.82</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>1258.HK</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>中国有色矿业</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>-21.51</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>0038.HK</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>第一拖拉机股份</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>-21.42</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>1117.HK</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>现代牧业</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>-21.39</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2382.HK</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>舜宇光学科技</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>-20.51</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>57.15</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>3759.HK</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>康龙化成</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>-20.26</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>1860.HK</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>汇量科技</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E11" s="10" t="n">
-        <v>-22.13</v>
-      </c>
-      <c r="F11" s="10" t="n">
+      <c r="E16" s="10" t="n">
+        <v>-19.84</v>
+      </c>
+      <c r="F16" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="10" t="n">
-        <v>10.52</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>1258.HK</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>中国有色矿业</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>-21.91</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>13.83</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>0038.HK</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>第一拖拉机股份</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>-21.78</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>7.665</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>1117.HK</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>现代牧业</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>-21.1</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>1.365</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>2382.HK</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>舜宇光学科技</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>-21</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>56.8</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>3759.HK</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>康龙化成</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>-20.56</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>26.9</v>
+      <c r="G16" s="10" t="n">
+        <v>10.83</v>
       </c>
     </row>
     <row r="17">
@@ -1980,13 +2249,13 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-19.94</v>
+        <v>-19.01</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>4.295</v>
+        <v>4.345</v>
       </c>
     </row>
     <row r="18">
@@ -2011,199 +2280,199 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-16.17</v>
+        <v>-17.28</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>143.1</v>
+        <v>141.2</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2269.HK</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>药明生物</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>-15.99</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>48.64</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>0999.HK</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>小菜园</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>-15.46</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>2419.HK</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>德康农牧</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E19" s="7" t="n">
-        <v>-15.4</v>
-      </c>
-      <c r="F19" s="7" t="n">
+      <c r="E21" s="7" t="n">
+        <v>-15.32</v>
+      </c>
+      <c r="F21" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="7" t="n">
-        <v>52.45</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>2269.HK</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>药明生物</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="G21" s="7" t="n">
+        <v>52.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>2202.HK</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>万科企业</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>-15.3</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>2.38</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>9688.HK</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>再鼎医药</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Health Care</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E20" s="5" t="n">
-        <v>-15.3</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>49.04</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>9688.HK</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>再鼎医药</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="E23" s="5" t="n">
+        <v>-15.17</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>17.95</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>1866.HK</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>中国心连心化肥</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E21" s="5" t="n">
-        <v>-15.22</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>17.94</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>1866.HK</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>中国心连心化肥</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="n">
-        <v>-15.17</v>
-      </c>
-      <c r="F22" s="9" t="n">
+      <c r="E24" s="9" t="n">
+        <v>-14.27</v>
+      </c>
+      <c r="F24" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="9" t="n">
-        <v>9.84</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>2202.HK</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>万科企业</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>-14.23</v>
-      </c>
-      <c r="F23" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G23" s="8" t="n">
-        <v>2.41</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>0999.HK</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>小菜园</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>-13.75</v>
-      </c>
-      <c r="F24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="3" t="n">
-        <v>8.06</v>
+      <c r="G24" s="9" t="n">
+        <v>9.945</v>
       </c>
     </row>
     <row r="25">
@@ -2228,24 +2497,24 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>-11.67</v>
+        <v>-11.97</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>2</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>8.895</v>
+        <v>8.865</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>1177.HK</t>
+          <t>3347.HK</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>中国生物制药</t>
+          <t>泰格医药</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -2259,24 +2528,24 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>-11.32</v>
+        <v>-11.66</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>5.25</v>
+        <v>41.66</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>3347.HK</t>
+          <t>1177.HK</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>泰格医药</t>
+          <t>中国生物制药</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -2290,13 +2559,13 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-11.32</v>
+        <v>-10.98</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>41.82</v>
+        <v>5.27</v>
       </c>
     </row>
     <row r="28">
@@ -2321,13 +2590,13 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>-9.619999999999999</v>
+        <v>-9.130000000000001</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>1.88</v>
+        <v>1.89</v>
       </c>
     </row>
     <row r="29">
@@ -2352,106 +2621,106 @@
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>-8.33</v>
+        <v>-8.23</v>
       </c>
       <c r="F29" s="5" t="n">
         <v>2</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>200.4</v>
+        <v>200.6</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>0013.HK</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>和黄医药</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>-6.78</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>21.44</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>0308.HK</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>香港中旅</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>A·PULLBACK 🟡</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>-6.51</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>2357.HK</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>中航科工</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>A·PULLBACK 🟡</t>
         </is>
       </c>
-      <c r="E30" s="2" t="n">
-        <v>-6.66</v>
-      </c>
-      <c r="F30" s="2" t="n">
+      <c r="E32" s="2" t="n">
+        <v>-6.04</v>
+      </c>
+      <c r="F32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="2" t="n">
-        <v>3.015</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>0013.HK</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>和黄医药</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="n">
-        <v>-6.61</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G31" s="5" t="n">
-        <v>21.48</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>0308.HK</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>香港中旅</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>A·PULLBACK 🟡</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>-6.51</v>
-      </c>
-      <c r="F32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="3" t="n">
-        <v>1.14</v>
+      <c r="G32" s="2" t="n">
+        <v>3.035</v>
       </c>
     </row>
     <row r="33">
@@ -2509,7 +2778,7 @@
         <v>4</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>17.41</v>
+        <v>17.53</v>
       </c>
     </row>
     <row r="35">
@@ -2538,7 +2807,7 @@
         <v>3</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>16.1</v>
+        <v>16.23</v>
       </c>
     </row>
     <row r="36">
@@ -2567,7 +2836,7 @@
         <v>4</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>11.1</v>
+        <v>11.16</v>
       </c>
     </row>
     <row r="37">
@@ -2596,7 +2865,7 @@
         <v>4</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>30.2</v>
+        <v>30.06</v>
       </c>
     </row>
     <row r="38">
@@ -2625,7 +2894,7 @@
         <v>4</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>1.215</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="39">
@@ -2654,7 +2923,7 @@
         <v>4</v>
       </c>
       <c r="G39" s="11" t="n">
-        <v>29.9</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="40">
@@ -2683,7 +2952,7 @@
         <v>4</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>4.735</v>
+        <v>4.76</v>
       </c>
     </row>
     <row r="41">
@@ -2712,7 +2981,7 @@
         <v>1</v>
       </c>
       <c r="G41" s="11" t="n">
-        <v>5.33</v>
+        <v>5.345</v>
       </c>
     </row>
     <row r="42">
@@ -2741,7 +3010,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>75.2</v>
+        <v>75.45</v>
       </c>
     </row>
     <row r="43">
@@ -2770,7 +3039,7 @@
         <v>4</v>
       </c>
       <c r="G43" s="10" t="n">
-        <v>28.48</v>
+        <v>28.58</v>
       </c>
     </row>
     <row r="44">
@@ -2799,7 +3068,7 @@
         <v>2</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>14.88</v>
+        <v>15.03</v>
       </c>
     </row>
     <row r="45">
@@ -2828,7 +3097,7 @@
         <v>3</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>34.76</v>
+        <v>34</v>
       </c>
     </row>
     <row r="46">
@@ -2857,7 +3126,7 @@
         <v>4</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>4.385</v>
+        <v>4.39</v>
       </c>
     </row>
     <row r="47">
@@ -2886,7 +3155,7 @@
         <v>2</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>21</v>
+        <v>20.44</v>
       </c>
     </row>
     <row r="48">
@@ -2915,18 +3184,18 @@
         <v>4</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>307.6</v>
+        <v>311.6</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>9896.HK</t>
+          <t>1928.HK</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>名创优品</t>
+          <t>金沙中国有限公司</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2941,21 +3210,21 @@
       </c>
       <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>20.42</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>1928.HK</t>
+          <t>1128.HK</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>金沙中国有限公司</t>
+          <t>永利澳门</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -2973,47 +3242,47 @@
         <v>4</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>11.17</v>
+        <v>4.98</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>1128.HK</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>永利澳门</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G51" s="3" t="n">
-        <v>4.99</v>
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>9980.HK</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>东鹏饮料</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr"/>
+      <c r="F51" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>95.65000000000001</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>9980.HK</t>
+          <t>2367.HK</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>东鹏饮料</t>
+          <t>巨子生物</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
@@ -3028,50 +3297,50 @@
       </c>
       <c r="E52" s="7" t="inlineStr"/>
       <c r="F52" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G52" s="7" t="n">
-        <v>95.2</v>
+        <v>23.22</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>2367.HK</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>巨子生物</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
-        <is>
-          <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr"/>
-      <c r="F53" s="7" t="n">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>6936.HK</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>顺丰控股</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G53" s="7" t="n">
-        <v>22.96</v>
+      <c r="G53" s="2" t="n">
+        <v>28.34</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>6936.HK</t>
+          <t>0066.HK</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>顺丰控股</t>
+          <t>港铁公司</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3086,21 +3355,21 @@
       </c>
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>28.48</v>
+        <v>31.86</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>0066.HK</t>
+          <t>0669.HK</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>港铁公司</t>
+          <t>创科实业</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3118,76 +3387,76 @@
         <v>2</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>31.72</v>
+        <v>128.1</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>0669.HK</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>创科实业</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G56" s="2" t="n">
-        <v>128.2</v>
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>1818.HK</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>招金矿业</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr"/>
+      <c r="F56" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G56" s="9" t="n">
+        <v>17.41</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="9" t="inlineStr">
-        <is>
-          <t>1818.HK</t>
-        </is>
-      </c>
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>招金矿业</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E57" s="9" t="inlineStr"/>
-      <c r="F57" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="G57" s="9" t="n">
-        <v>17.18</v>
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>9903.HK</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>天数智芯</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>79.8</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>9903.HK</t>
+          <t>0501.HK</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>天数智芯</t>
+          <t>豪威集团</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3202,10 +3471,10 @@
       </c>
       <c r="E58" s="4" t="inlineStr"/>
       <c r="F58" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>81</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="59">
@@ -3234,18 +3503,18 @@
         <v>4</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>26.96</v>
+        <v>27.08</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>0501.HK</t>
+          <t>2676.HK</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>豪威集团</t>
+          <t>纳芯微</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3260,50 +3529,50 @@
       </c>
       <c r="E60" s="4" t="inlineStr"/>
       <c r="F60" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>63.25</v>
+        <v>136</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>2676.HK</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>纳芯微</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr"/>
-      <c r="F61" s="4" t="n">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>1801.HK</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>信达生物</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Health Care</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr"/>
+      <c r="F61" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="G61" s="4" t="n">
-        <v>140.5</v>
+      <c r="G61" s="5" t="n">
+        <v>87.75</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>1801.HK</t>
+          <t>3696.HK</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>信达生物</t>
+          <t>英矽智能</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -3321,18 +3590,18 @@
         <v>2</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>87.7</v>
+        <v>37.64</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>3696.HK</t>
+          <t>3692.HK</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>英矽智能</t>
+          <t>翰森制药</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -3347,108 +3616,108 @@
       </c>
       <c r="E63" s="5" t="inlineStr"/>
       <c r="F63" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G63" s="5" t="n">
+        <v>31.38</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>2889.HK</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>博泰车联</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr"/>
+      <c r="F64" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>58.9</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>6818.HK</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>中国光大银行</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr"/>
+      <c r="F65" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G65" s="6" t="n">
+        <v>2.81</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>7687.HK</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>易控智驾</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G63" s="5" t="n">
-        <v>37.98</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
-        <is>
-          <t>3692.HK</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>翰森制药</t>
-        </is>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>Health Care</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="inlineStr"/>
-      <c r="F64" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G64" s="5" t="n">
-        <v>31.42</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>2889.HK</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>博泰车联</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr"/>
-      <c r="F65" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G65" s="3" t="n">
-        <v>58.85</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>6818.HK</t>
-        </is>
-      </c>
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>中国光大银行</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D66" s="6" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr"/>
-      <c r="F66" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G66" s="6" t="n">
-        <v>2.775</v>
+      <c r="G66" s="4" t="n">
+        <v>64.7</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>7687.HK</t>
+          <t>6880.HK</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>易控智驾</t>
+          <t>MOMENTA-W</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3463,39 +3732,39 @@
       </c>
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>64.25</v>
+        <v>163.8</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>6880.HK</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>MOMENTA-W</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>B·EXIT 🔴</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr"/>
-      <c r="F68" s="4" t="n">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t>1033.HK</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>中石化油服</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
+        <is>
+          <t>B·EXIT 🔴</t>
+        </is>
+      </c>
+      <c r="E68" s="12" t="inlineStr"/>
+      <c r="F68" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G68" s="4" t="n">
-        <v>157.4</v>
+      <c r="G68" s="12" t="n">
+        <v>0.615</v>
       </c>
     </row>
     <row r="69">
@@ -3524,7 +3793,7 @@
         <v>1</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>2.9</v>
+        <v>2.925</v>
       </c>
     </row>
     <row r="70">
@@ -3553,7 +3822,7 @@
         <v>4</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>1.055</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="71">
@@ -3582,7 +3851,7 @@
         <v>4</v>
       </c>
       <c r="G71" s="5" t="n">
-        <v>11.22</v>
+        <v>11.25</v>
       </c>
     </row>
     <row r="72">
@@ -3611,7 +3880,7 @@
         <v>1</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>15.63</v>
+        <v>15.65</v>
       </c>
     </row>
     <row r="73">
@@ -3640,7 +3909,7 @@
         <v>1</v>
       </c>
       <c r="G73" s="5" t="n">
-        <v>63.95</v>
+        <v>64.75</v>
       </c>
     </row>
     <row r="74">
@@ -3669,7 +3938,7 @@
         <v>4</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>38.4</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="75">
@@ -3698,7 +3967,7 @@
         <v>3</v>
       </c>
       <c r="G75" s="5" t="n">
-        <v>9.85</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="76">
@@ -3727,7 +3996,7 @@
         <v>3</v>
       </c>
       <c r="G76" s="5" t="n">
-        <v>6.735</v>
+        <v>6.675</v>
       </c>
     </row>
     <row r="77">
@@ -3756,7 +4025,7 @@
         <v>1</v>
       </c>
       <c r="G77" s="10" t="n">
-        <v>12.12</v>
+        <v>12.23</v>
       </c>
     </row>
     <row r="78">
@@ -3785,7 +4054,7 @@
         <v>3</v>
       </c>
       <c r="G78" s="11" t="n">
-        <v>1.6</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="79">
@@ -3814,69 +4083,69 @@
         <v>1</v>
       </c>
       <c r="G79" s="11" t="n">
-        <v>0.985</v>
+        <v>0.995</v>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="9" t="inlineStr">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>3887.HK</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>HASHKEY HLDGS</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>C·PULLBACK 🟠</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="n">
+        <v>-33.67</v>
+      </c>
+      <c r="F80" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G80" s="6" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="inlineStr">
         <is>
           <t>3330.HK</t>
         </is>
       </c>
-      <c r="B80" s="9" t="inlineStr">
+      <c r="B81" s="9" t="inlineStr">
         <is>
           <t>灵宝黄金</t>
         </is>
       </c>
-      <c r="C80" s="9" t="inlineStr">
+      <c r="C81" s="9" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="D80" s="9" t="inlineStr">
+      <c r="D81" s="9" t="inlineStr">
         <is>
           <t>C·PULLBACK 🟠</t>
         </is>
       </c>
-      <c r="E80" s="9" t="n">
-        <v>-33.02</v>
-      </c>
-      <c r="F80" s="9" t="n">
+      <c r="E81" s="9" t="n">
+        <v>-32.9</v>
+      </c>
+      <c r="F81" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="G80" s="9" t="n">
-        <v>16.88</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="6" t="inlineStr">
-        <is>
-          <t>3887.HK</t>
-        </is>
-      </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>HASHKEY HLDGS</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D81" s="6" t="inlineStr">
-        <is>
-          <t>C·PULLBACK 🟠</t>
-        </is>
-      </c>
-      <c r="E81" s="6" t="n">
-        <v>-32.82</v>
-      </c>
-      <c r="F81" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="G81" s="6" t="n">
-        <v>1.975</v>
+      <c r="G81" s="9" t="n">
+        <v>16.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
trend screener update 2026-10-15 14:12 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -3451,12 +3451,12 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>0501.HK</t>
+          <t>1810.HK</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>豪威集团</t>
+          <t>小米集团-W</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3474,18 +3474,18 @@
         <v>4</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>63.4</v>
+        <v>27.08</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>1810.HK</t>
+          <t>2676.HK</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>小米集团-W</t>
+          <t>纳芯微</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3500,21 +3500,21 @@
       </c>
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>27.08</v>
+        <v>136</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>2676.HK</t>
+          <t>0501.HK</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>纳芯微</t>
+          <t>豪威集团</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3529,10 +3529,10 @@
       </c>
       <c r="E60" s="4" t="inlineStr"/>
       <c r="F60" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>136</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="61">

</xml_diff>

<commit_message>
trend screener update 2026-10-15 14:37 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -3683,12 +3683,12 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>7687.HK</t>
+          <t>6880.HK</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>易控智驾</t>
+          <t>MOMENTA-W</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -3703,21 +3703,21 @@
       </c>
       <c r="E66" s="4" t="inlineStr"/>
       <c r="F66" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>64.7</v>
+        <v>163.8</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>6880.HK</t>
+          <t>7687.HK</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>MOMENTA-W</t>
+          <t>易控智驾</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3732,10 +3732,10 @@
       </c>
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>163.8</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="68">
@@ -3770,12 +3770,12 @@
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>0151.HK</t>
+          <t>1610.HK</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>中国旺旺</t>
+          <t>中粮家佳康</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
@@ -3790,21 +3790,21 @@
       </c>
       <c r="E69" s="7" t="inlineStr"/>
       <c r="F69" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>2.925</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>1610.HK</t>
+          <t>0151.HK</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>中粮家佳康</t>
+          <t>中国旺旺</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
@@ -3819,10 +3819,10 @@
       </c>
       <c r="E70" s="7" t="inlineStr"/>
       <c r="F70" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>1.06</v>
+        <v>2.925</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
trend screener update 2026-10-15 17:18 UTC
</commit_message>
<xml_diff>
--- a/data/v5_4_hk.xlsx
+++ b/data/v5_4_hk.xlsx
@@ -3451,12 +3451,12 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>1810.HK</t>
+          <t>0501.HK</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>小米集团-W</t>
+          <t>豪威集团</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3474,18 +3474,18 @@
         <v>4</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>27.08</v>
+        <v>63.4</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>2676.HK</t>
+          <t>1810.HK</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>纳芯微</t>
+          <t>小米集团-W</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3500,21 +3500,21 @@
       </c>
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>136</v>
+        <v>27.08</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>0501.HK</t>
+          <t>2676.HK</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>豪威集团</t>
+          <t>纳芯微</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3529,10 +3529,10 @@
       </c>
       <c r="E60" s="4" t="inlineStr"/>
       <c r="F60" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>63.4</v>
+        <v>136</v>
       </c>
     </row>
     <row r="61">
@@ -3683,12 +3683,12 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>6880.HK</t>
+          <t>7687.HK</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>MOMENTA-W</t>
+          <t>易控智驾</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -3703,21 +3703,21 @@
       </c>
       <c r="E66" s="4" t="inlineStr"/>
       <c r="F66" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>163.8</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>7687.HK</t>
+          <t>6880.HK</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>易控智驾</t>
+          <t>MOMENTA-W</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3732,10 +3732,10 @@
       </c>
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>64.7</v>
+        <v>163.8</v>
       </c>
     </row>
     <row r="68">
@@ -3770,12 +3770,12 @@
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>1610.HK</t>
+          <t>0151.HK</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>中粮家佳康</t>
+          <t>中国旺旺</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
@@ -3790,21 +3790,21 @@
       </c>
       <c r="E69" s="7" t="inlineStr"/>
       <c r="F69" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>1.06</v>
+        <v>2.925</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>0151.HK</t>
+          <t>1610.HK</t>
         </is>
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>中国旺旺</t>
+          <t>中粮家佳康</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
@@ -3819,10 +3819,10 @@
       </c>
       <c r="E70" s="7" t="inlineStr"/>
       <c r="F70" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G70" s="7" t="n">
-        <v>2.925</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="71">
@@ -3857,12 +3857,12 @@
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>1099.HK</t>
+          <t>2506.HK</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>国药控股</t>
+          <t>讯飞医疗科技</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -3880,18 +3880,18 @@
         <v>1</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>15.65</v>
+        <v>64.75</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>2506.HK</t>
+          <t>1099.HK</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>讯飞医疗科技</t>
+          <t>国药控股</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -3909,7 +3909,7 @@
         <v>1</v>
       </c>
       <c r="G73" s="5" t="n">
-        <v>64.75</v>
+        <v>15.65</v>
       </c>
     </row>
     <row r="74">

</xml_diff>